<commit_message>
feat: paliers de difficulté des questions et 40 questions de la zone 1 (paliers 2 et 3)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e2e/fixtures/import-e2e.xlsx
+++ b/e2e/fixtures/import-e2e.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t xml:space="preserve">Zone</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t xml:space="preserve">Note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Palier</t>
   </si>
   <si>
     <t xml:space="preserve">[E2E import] Première question</t>
@@ -130,6 +133,7 @@
     <col min="7" max="7" width="30" customWidth="1"/>
     <col min="8" max="8" width="30" customWidth="1"/>
     <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="10" max="10" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -160,25 +164,28 @@
       <c r="I1" t="s" s="1">
         <v>8</v>
       </c>
+      <c r="J1" t="s" s="1">
+        <v>9</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -186,10 +193,10 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -197,10 +204,10 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -208,7 +215,7 @@
         <v>0</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
         <v>2</v>
@@ -219,10 +226,10 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>